<commit_message>
Added Digital Function settings
</commit_message>
<xml_diff>
--- a/d890uv/Tracking CPS-Menu.xlsx
+++ b/d890uv/Tracking CPS-Menu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andreas\Documents\codeplugs\d890uv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3122EC6D-A5D3-4235-B6DF-6727BF61452B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE54D5E3-C0C8-4CB6-81D5-B508EBF16808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9012" yWindow="456" windowWidth="12240" windowHeight="11472" xr2:uid="{BBF6BA9B-FEA4-4E33-A5D2-E76637C1E8DB}"/>
   </bookViews>
@@ -921,7 +921,7 @@
         <v>47</v>
       </c>
       <c r="E30" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Added ARC4 keys/bitmap and AES bitmap
</commit_message>
<xml_diff>
--- a/d890uv/Tracking CPS-Menu.xlsx
+++ b/d890uv/Tracking CPS-Menu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andreas\Documents\codeplugs\d890uv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE54D5E3-C0C8-4CB6-81D5-B508EBF16808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C31AF47F-FA25-41CF-AA25-131C74B56851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9012" yWindow="456" windowWidth="12240" windowHeight="11472" xr2:uid="{BBF6BA9B-FEA4-4E33-A5D2-E76637C1E8DB}"/>
   </bookViews>
@@ -1063,7 +1063,7 @@
         <v>47</v>
       </c>
       <c r="E44" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="45" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Added DMR callsign database
</commit_message>
<xml_diff>
--- a/d890uv/Tracking CPS-Menu.xlsx
+++ b/d890uv/Tracking CPS-Menu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andreas\Documents\codeplugs\d890uv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{304D3183-78EF-4F06-9B8D-4DE283A18A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{465EE304-457C-4696-A42E-A51468EBA9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10512" yWindow="60" windowWidth="12528" windowHeight="12180" xr2:uid="{BBF6BA9B-FEA4-4E33-A5D2-E76637C1E8DB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BBF6BA9B-FEA4-4E33-A5D2-E76637C1E8DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -1382,7 +1382,7 @@
         <v>47</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="55" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Fixed DMR callsign DB and finalized Roaming Zone/Channels
</commit_message>
<xml_diff>
--- a/d890uv/Tracking CPS-Menu.xlsx
+++ b/d890uv/Tracking CPS-Menu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andreas\Documents\codeplugs\d890uv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{465EE304-457C-4696-A42E-A51468EBA9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5802EFD-F7D8-43C2-97AF-31CD1C87B906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BBF6BA9B-FEA4-4E33-A5D2-E76637C1E8DB}"/>
   </bookViews>
@@ -1304,7 +1304,7 @@
         <v>47</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
     </row>
     <row r="49" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -1317,7 +1317,7 @@
         <v>47</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -1391,9 +1391,9 @@
         <v>41</v>
       </c>
       <c r="C55" s="6"/>
-      <c r="D55" s="7"/>
+      <c r="D55" s="11"/>
       <c r="E55" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="56" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">

</xml_diff>